<commit_message>
data: update VIN locations via web import
</commit_message>
<xml_diff>
--- a/VIN_To_LocationCode.xlsx
+++ b/VIN_To_LocationCode.xlsx
@@ -436,7 +436,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>KL</t>
+          <t>Test</t>
         </is>
       </c>
     </row>
@@ -2944,7 +2944,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>Test</t>
+          <t>test</t>
         </is>
       </c>
     </row>
@@ -2956,7 +2956,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>Stock</t>
+          <t>Test</t>
         </is>
       </c>
     </row>

</xml_diff>